<commit_message>
finilization of evaluation plots
</commit_message>
<xml_diff>
--- a/outputs/model_results/MCLR/Model 1_seuils.xlsx
+++ b/outputs/model_results/MCLR/Model 1_seuils.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-3.04</t>
+          <t>-3.03</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.494</t>
+          <t>0.467</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,14 +486,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-2.2</t>
+          <t>-2.3</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6613</v>
+        <v>6686</v>
       </c>
       <c r="G2" t="n">
-        <v>3216</v>
+        <v>3160</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0061</t>
+          <t>0.0057</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0043</t>
+          <t>0.0038</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.492</t>
+          <t>0.464</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6869</v>
+        <v>7022</v>
       </c>
       <c r="G3" t="n">
-        <v>3145</v>
+        <v>3436</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.0059</t>
+          <t>0.0055</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0041</t>
+          <t>0.0037</t>
         </is>
       </c>
     </row>
@@ -572,12 +572,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.493</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.14</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6813</v>
+        <v>7063</v>
       </c>
       <c r="G4" t="n">
-        <v>3333</v>
+        <v>3361</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.0055</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0037</t>
         </is>
       </c>
     </row>
@@ -615,17 +615,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.497</t>
+          <t>0.463</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6892</v>
+        <v>7148</v>
       </c>
       <c r="G5" t="n">
-        <v>3294</v>
+        <v>3329</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.0055</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0037</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test of various other models
</commit_message>
<xml_diff>
--- a/outputs/model_results/MCLR/Model 1_seuils.xlsx
+++ b/outputs/model_results/MCLR/Model 1_seuils.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-3.03</t>
+          <t>-3.02</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.467</t>
+          <t>0.485</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,14 +486,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-2.3</t>
+          <t>-2.2</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6686</v>
+        <v>6654</v>
       </c>
       <c r="G2" t="n">
-        <v>3160</v>
+        <v>3243</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0057</t>
+          <t>0.0059</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0042</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.464</t>
+          <t>0.482</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>7022</v>
+        <v>6349</v>
       </c>
       <c r="G3" t="n">
-        <v>3436</v>
+        <v>3308</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.0055</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0043</t>
         </is>
       </c>
     </row>
@@ -567,17 +567,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.463</t>
+          <t>0.485</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7063</v>
+        <v>6541</v>
       </c>
       <c r="G4" t="n">
-        <v>3361</v>
+        <v>3407</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.0055</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0042</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.463</t>
+          <t>0.485</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>7148</v>
+        <v>6684</v>
       </c>
       <c r="G5" t="n">
-        <v>3329</v>
+        <v>3460</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0055</t>
+          <t>0.0059</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0042</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update of encoding for MCLR models
</commit_message>
<xml_diff>
--- a/outputs/model_results/MCLR/Model 1_seuils.xlsx
+++ b/outputs/model_results/MCLR/Model 1_seuils.xlsx
@@ -471,17 +471,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-3.02</t>
+          <t>-2.93</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.485</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-3.8</t>
+          <t>-3.6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,10 +490,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6654</v>
+        <v>2016</v>
       </c>
       <c r="G2" t="n">
-        <v>3243</v>
+        <v>2351</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0059</t>
+          <t>0.0097</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0067</t>
         </is>
       </c>
     </row>
@@ -519,29 +519,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>-0.95</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.482</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-1.8</t>
+          <t>-1.7</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.24</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6349</v>
+        <v>2046</v>
       </c>
       <c r="G3" t="n">
-        <v>3308</v>
+        <v>2375</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.0096</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0043</t>
+          <t>0.0066</t>
         </is>
       </c>
     </row>
@@ -567,17 +567,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.485</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>6541</v>
+        <v>2093</v>
       </c>
       <c r="G4" t="n">
-        <v>3407</v>
+        <v>2425</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.0095</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0065</t>
         </is>
       </c>
     </row>
@@ -615,17 +615,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.485</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6684</v>
+        <v>2121</v>
       </c>
       <c r="G5" t="n">
-        <v>3460</v>
+        <v>2603</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0059</t>
+          <t>0.0094</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.0042</t>
+          <t>0.0064</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
integration of the MCLR models inside the benchmark pipline (only for the train test for now)
</commit_message>
<xml_diff>
--- a/outputs/model_results/MCLR/Model 1_seuils.xlsx
+++ b/outputs/model_results/MCLR/Model 1_seuils.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-2.93</t>
+          <t>-2.97</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-3.6</t>
+          <t>-3.7</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -490,10 +490,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2016</v>
+        <v>2409</v>
       </c>
       <c r="G2" t="n">
-        <v>2351</v>
+        <v>2685</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0097</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0067</t>
+          <t>0.0063</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-0.95</t>
+          <t>-0.98</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2046</v>
+        <v>2394</v>
       </c>
       <c r="G3" t="n">
-        <v>2375</v>
+        <v>2587</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.0096</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0066</t>
+          <t>0.0064</t>
         </is>
       </c>
     </row>
@@ -567,17 +567,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2093</v>
+        <v>2431</v>
       </c>
       <c r="G4" t="n">
-        <v>2425</v>
+        <v>2682</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.0095</t>
+          <t>0.0089</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0065</t>
+          <t>0.0063</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2121</v>
+        <v>2464</v>
       </c>
       <c r="G5" t="n">
-        <v>2603</v>
+        <v>2551</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0094</t>
+          <t>0.0089</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.0064</t>
+          <t>0.0063</t>
         </is>
       </c>
     </row>

</xml_diff>